<commit_message>
chore(samples): unique PDF per demo project via pdf-lib
- Add scripts/generate-project-sample-pdfs.mjs and public/samples/projects/proj-00x.pdf
- Point each DEMO_PROJECTS pdf_url to its own file; keep SAMPLE_TEAM_SUBMISSION_PDF as proj-001 example
- Refresh import CSV/XLSX; remove generic sample-submission.pdf; npm script generate-project-pdfs
</commit_message>
<xml_diff>
--- a/public/samples/organiser-projects-import.xlsx
+++ b/public/samples/organiser-projects-import.xlsx
@@ -421,7 +421,7 @@
         <v>Singapore</v>
       </c>
       <c r="C2" t="str">
-        <v>/samples/sample-submission.pdf</v>
+        <v>/samples/projects/proj-001.pdf</v>
       </c>
       <c r="D2" t="str">
         <v>https://www.youtube.com/watch?v=dQw4w9WgXcQ</v>
@@ -435,7 +435,7 @@
         <v>Malaysia</v>
       </c>
       <c r="C3" t="str">
-        <v>/samples/sample-submission.pdf</v>
+        <v>/samples/projects/proj-002.pdf</v>
       </c>
       <c r="D3" t="str">
         <v/>

</xml_diff>